<commit_message>
fix: sostituisci width=True con use_container_width=True (Streamlit API)
- app.py: Logout button
- albero_dipendenze.py: st.dataframe
- dashboard.py: st.plotly_chart (2 occorrenze)

width non è parametro valido in Streamlit - use_container_width è il corretto.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/part_numbers_db.xlsx
+++ b/data/part_numbers_db.xlsx
@@ -7235,7 +7235,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>2026-03-01 20:17:44</t>
+          <t>2026-03-01 21:15:59</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -7398,7 +7398,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>2026-03-01 20:17:45</t>
+          <t>2026-03-01 21:15:59</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -7556,7 +7556,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>2026-03-01 20:17:46</t>
+          <t>2026-03-01 21:16:00</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -7704,7 +7704,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>2026-03-01 20:17:47</t>
+          <t>2026-03-01 21:16:01</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -7862,7 +7862,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>2026-03-01 20:17:48</t>
+          <t>2026-03-01 21:16:02</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -8010,7 +8010,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>2026-03-01 20:17:49</t>
+          <t>2026-03-01 21:16:03</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -8153,7 +8153,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>2026-03-01 20:17:50</t>
+          <t>2026-03-01 21:16:03</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -8311,7 +8311,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>2026-03-01 20:17:51</t>
+          <t>2026-03-01 21:16:04</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -8459,7 +8459,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>2026-03-01 20:17:52</t>
+          <t>2026-03-01 21:16:05</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -8602,7 +8602,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>2026-03-01 20:17:53</t>
+          <t>2026-03-01 21:16:06</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -8750,7 +8750,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>2026-03-01 20:17:53</t>
+          <t>2026-03-01 21:16:06</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -8903,7 +8903,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>2026-03-01 20:17:54</t>
+          <t>2026-03-01 21:16:07</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -9051,7 +9051,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>2026-03-01 20:17:55</t>
+          <t>2026-03-01 21:16:08</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -9189,7 +9189,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>2026-03-01 20:17:55</t>
+          <t>2026-03-01 21:16:09</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -9332,7 +9332,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>2026-03-01 20:17:56</t>
+          <t>2026-03-01 21:16:09</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">

</xml_diff>

<commit_message>
fix: sostituisci TUTTI i width=True con use_container_width=True (Streamlit API)
Replacement globale in src/tabs/:
- st.dataframe: 14 occorrenze
- st.plotly_chart: 5 occorrenze
- st.button: 1 occorrenza

width non è parametro valido in Streamlit - use_container_width è il corretto.

Questo assicura che tutti i grafici e le tabelle occupino la larghezza del container correttamente.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/part_numbers_db.xlsx
+++ b/data/part_numbers_db.xlsx
@@ -7235,7 +7235,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>2026-03-01 21:15:59</t>
+          <t>2026-03-01 21:20:42</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -7398,7 +7398,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>2026-03-01 21:15:59</t>
+          <t>2026-03-01 21:20:43</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -7556,7 +7556,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>2026-03-01 21:16:00</t>
+          <t>2026-03-01 21:20:43</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -7704,7 +7704,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>2026-03-01 21:16:01</t>
+          <t>2026-03-01 21:20:44</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -7862,7 +7862,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>2026-03-01 21:16:02</t>
+          <t>2026-03-01 21:20:45</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -8010,7 +8010,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>2026-03-01 21:16:03</t>
+          <t>2026-03-01 21:20:46</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -8153,7 +8153,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>2026-03-01 21:16:03</t>
+          <t>2026-03-01 21:20:47</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -8311,7 +8311,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>2026-03-01 21:16:04</t>
+          <t>2026-03-01 21:20:47</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -8459,7 +8459,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>2026-03-01 21:16:05</t>
+          <t>2026-03-01 21:20:48</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -8602,7 +8602,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>2026-03-01 21:16:06</t>
+          <t>2026-03-01 21:20:49</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -8750,7 +8750,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>2026-03-01 21:16:06</t>
+          <t>2026-03-01 21:20:50</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -8903,7 +8903,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>2026-03-01 21:16:07</t>
+          <t>2026-03-01 21:20:51</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -9051,7 +9051,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>2026-03-01 21:16:08</t>
+          <t>2026-03-01 21:20:51</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -9189,7 +9189,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>2026-03-01 21:16:09</t>
+          <t>2026-03-01 21:20:52</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -9332,7 +9332,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>2026-03-01 21:16:09</t>
+          <t>2026-03-01 21:20:53</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">

</xml_diff>

<commit_message>
fix: ripulisci doppi use_container_use_container_width
Rimosso prefisso duplicato causato da sostituzione multiple.
Tutti i st.dataframe e st.plotly_chart ora usano use_container_width correttamente.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/part_numbers_db.xlsx
+++ b/data/part_numbers_db.xlsx
@@ -7235,7 +7235,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>2026-03-01 21:20:42</t>
+          <t>2026-03-01 21:23:57</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -7398,7 +7398,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>2026-03-01 21:20:43</t>
+          <t>2026-03-01 21:23:57</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -7556,7 +7556,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>2026-03-01 21:20:43</t>
+          <t>2026-03-01 21:23:58</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -7704,7 +7704,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>2026-03-01 21:20:44</t>
+          <t>2026-03-01 21:23:58</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -7862,7 +7862,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>2026-03-01 21:20:45</t>
+          <t>2026-03-01 21:23:59</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -8010,7 +8010,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>2026-03-01 21:20:46</t>
+          <t>2026-03-01 21:24:00</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -8153,7 +8153,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>2026-03-01 21:20:47</t>
+          <t>2026-03-01 21:24:00</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -8311,7 +8311,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>2026-03-01 21:20:47</t>
+          <t>2026-03-01 21:24:01</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -8459,7 +8459,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>2026-03-01 21:20:48</t>
+          <t>2026-03-01 21:24:02</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -8602,7 +8602,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>2026-03-01 21:20:49</t>
+          <t>2026-03-01 21:24:03</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -8750,7 +8750,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>2026-03-01 21:20:50</t>
+          <t>2026-03-01 21:24:04</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -8903,7 +8903,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>2026-03-01 21:20:51</t>
+          <t>2026-03-01 21:24:04</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -9051,7 +9051,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>2026-03-01 21:20:51</t>
+          <t>2026-03-01 21:24:05</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -9189,7 +9189,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>2026-03-01 21:20:52</t>
+          <t>2026-03-01 21:24:06</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -9332,7 +9332,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>2026-03-01 21:20:53</t>
+          <t>2026-03-01 21:24:07</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">

</xml_diff>